<commit_message>
Implemented refund can cancel payemnt
</commit_message>
<xml_diff>
--- a/docs/gini-flow/billing-template.xlsx
+++ b/docs/gini-flow/billing-template.xlsx
@@ -559,7 +559,7 @@
     <t>Follow Up</t>
   </si>
   <si>
-    <t>Test items only (required for them): the test's name exactly as in the test catalogue list you were given.</t>
+    <t>Test items only (required for them): the test's name exactly as in Scribe's test catalogue. A test that is only in the lab report catalogue must be added to the test catalogue by an admin first.</t>
   </si>
   <si>
     <t>not a test item</t>
@@ -2789,7 +2789,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="62" ht="33" customHeight="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" ht="48" customHeight="1" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
         <v>154</v>
       </c>

</xml_diff>

<commit_message>
Redesign the ui and updated
</commit_message>
<xml_diff>
--- a/docs/gini-flow/billing-template.xlsx
+++ b/docs/gini-flow/billing-template.xlsx
@@ -361,7 +361,7 @@
     <t>Gini Scribe — billing data template</t>
   </si>
   <si>
-    <t>Fill the sheets, then upload the file in Settings › Billing › Bulk import. Nothing is saved until every row passes the checks.</t>
+    <t>Fill the sheets, then upload the file in Settings › Billing › Bulk import. Every row is checked and listed as Ready, Needs override, Failed or Unchanged; nothing is saved until you press Commit.</t>
   </si>
   <si>
     <t>How to fill this file</t>
@@ -466,7 +466,7 @@
     <t>Rule 16</t>
   </si>
   <si>
-    <t>Any error stops the whole upload: fix the rows listed in the error file and upload again.</t>
+    <t>A row with an error fails and is skipped, and so is every new row that depends on it; the other rows can still be saved. A change to a row already in Scribe is saved only if you choose Override for it — otherwise the row is kept as it is. Download the failed rows, fix them and upload that file again.</t>
   </si>
   <si>
     <t>Allowed values</t>
@@ -2064,7 +2064,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="21" ht="33" customHeight="1" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" ht="78" customHeight="1" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>115</v>
       </c>

</xml_diff>

<commit_message>
Implemented cancel and restore the test
</commit_message>
<xml_diff>
--- a/docs/gini-flow/billing-template.xlsx
+++ b/docs/gini-flow/billing-template.xlsx
@@ -400,7 +400,7 @@
     <t>Rule 5</t>
   </si>
   <si>
-    <t>There are no packages. Each ordered test is always billed on its own line at its own price.</t>
+    <t>Each ordered test is always billed on its own line. A package (e.g. ABI + VPT at one combined price) is an automatic discount set up on the Discounts page, not an import row.</t>
   </si>
   <si>
     <t>Rule 6</t>
@@ -1811,7 +1811,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="10" ht="33" customHeight="1" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="48" customHeight="1" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>115</v>
       </c>

</xml_diff>